<commit_message>
Refine workbook count formulas and reviewer navigation
</commit_message>
<xml_diff>
--- a/verification/qualified-records.xlsx
+++ b/verification/qualified-records.xlsx
@@ -19992,7 +19992,7 @@
         <x:v>Table</x:v>
       </x:c>
       <x:c r="C5" s="78" t="n">
-        <x:f t="shared" ref="C5:C10" si="0">COUNTA(A12:A20)</x:f>
+        <x:f t="shared" ref="C5:C10" si="0">COUNTIFS($B$12:$B$39,$A5,$C$12:$C$39,$B5)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D5" s="79" t="n">
@@ -20020,7 +20020,7 @@
         <x:v>0.004736302539263777</x:v>
       </x:c>
       <x:c r="J5" s="78" t="n">
-        <x:f>SUM(E12:E20)</x:f>
+        <x:f>SUMIFS($E$12:$E$39,$B$12:$B$39,$A5,$C$12:$C$39,$B5)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="K5" s="59"/>
@@ -20034,7 +20034,7 @@
         <x:v>Table</x:v>
       </x:c>
       <x:c r="C6" s="96" t="n">
-        <x:f t="shared" si="0">COUNTA(A21:A21)</x:f>
+        <x:f t="shared" si="0">COUNTIFS($B$12:$B$39,$A6,$C$12:$C$39,$B6)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D6" s="97" t="n">
@@ -20062,7 +20062,7 @@
         <x:v>-0.00798611111111111</x:v>
       </x:c>
       <x:c r="J6" s="96" t="n">
-        <x:f>SUM(E21:E21)</x:f>
+        <x:f>SUMIFS($E$12:$E$39,$B$12:$B$39,$A6,$C$12:$C$39,$B6)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="K6" s="59"/>
@@ -20076,7 +20076,7 @@
         <x:v>Table</x:v>
       </x:c>
       <x:c r="C7" s="78" t="n">
-        <x:f t="shared" si="0">COUNTA(A22:A30)</x:f>
+        <x:f t="shared" si="0">COUNTIFS($B$12:$B$39,$A7,$C$12:$C$39,$B7)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D7" s="79" t="n">
@@ -20104,7 +20104,7 @@
         <x:v>0.022409309788321164</x:v>
       </x:c>
       <x:c r="J7" s="78" t="n">
-        <x:f>SUM(E22:E30)</x:f>
+        <x:f>SUMIFS($E$12:$E$39,$B$12:$B$39,$A7,$C$12:$C$39,$B7)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="K7" s="59"/>
@@ -20118,7 +20118,7 @@
         <x:v>Table</x:v>
       </x:c>
       <x:c r="C8" s="78" t="n">
-        <x:f t="shared" si="0">COUNTA(A31:A39)</x:f>
+        <x:f t="shared" si="0">COUNTIFS($B$12:$B$39,$A8,$C$12:$C$39,$B8)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D8" s="79" t="n">
@@ -20146,7 +20146,7 @@
         <x:v>0.028084267072685014</x:v>
       </x:c>
       <x:c r="J8" s="78" t="n">
-        <x:f>SUM(E31:E39)</x:f>
+        <x:f>SUMIFS($E$12:$E$39,$B$12:$B$39,$A8,$C$12:$C$39,$B8)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="K8" s="59"/>
@@ -20155,9 +20155,7 @@
     <x:row r="9">
       <x:c r="A9" s="20"/>
       <x:c r="B9" s="20"/>
-      <x:c r="C9" s="21">
-        <x:f t="shared" si="0"/>
-      </x:c>
+      <x:c r="C9" s="21"/>
       <x:c r="D9" s="22"/>
       <x:c r="E9" s="22"/>
       <x:c r="F9" s="22"/>
@@ -22460,7 +22458,7 @@
         <x:v>No Table</x:v>
       </x:c>
       <x:c r="C65" s="80" t="n">
-        <x:f>COUNTA(A43:A51)</x:f>
+        <x:f>COUNTIFS($B$43:$B$60,$A65,$C$43:$C$60,$B65)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D65" s="79" t="n">
@@ -22488,7 +22486,7 @@
         <x:v>0.01262964860193241</x:v>
       </x:c>
       <x:c r="J65" s="80" t="n">
-        <x:f>SUM(E43:E51)</x:f>
+        <x:f>SUMIFS($E$43:$E$60,$B$43:$B$60,$A65,$C$43:$C$60,$B65)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="K65" s="59"/>
@@ -22502,7 +22500,7 @@
         <x:v>No Table</x:v>
       </x:c>
       <x:c r="C66" s="80" t="n">
-        <x:f>COUNTA(A52:A60)</x:f>
+        <x:f>COUNTIFS($B$43:$B$60,$A66,$C$43:$C$60,$B66)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D66" s="79" t="n">
@@ -22530,7 +22528,7 @@
         <x:v>0.036938920579677965</x:v>
       </x:c>
       <x:c r="J66" s="80" t="n">
-        <x:f>SUM(E52:E60)</x:f>
+        <x:f>SUMIFS($E$43:$E$60,$B$43:$B$60,$A66,$C$43:$C$60,$B66)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="K66" s="59"/>

</xml_diff>